<commit_message>
Updated clusters with 2 PCA
</commit_message>
<xml_diff>
--- a/MASTER/cluster_plots_loadings/1995/pca_results_1995.xlsx
+++ b/MASTER/cluster_plots_loadings/1995/pca_results_1995.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,11 +444,6 @@
           <t>PC2</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>PC3</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -462,9 +457,6 @@
       <c r="C2" t="n">
         <v>0.1743457149584367</v>
       </c>
-      <c r="D2" t="n">
-        <v>0.633151850812806</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -478,9 +470,6 @@
       <c r="C3" t="n">
         <v>0.06723050390707017</v>
       </c>
-      <c r="D3" t="n">
-        <v>0.002803927787755511</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -494,9 +483,6 @@
       <c r="C4" t="n">
         <v>0.007877734388425772</v>
       </c>
-      <c r="D4" t="n">
-        <v>-0.004631330211285094</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -510,9 +496,6 @@
       <c r="C5" t="n">
         <v>0.4642250012442724</v>
       </c>
-      <c r="D5" t="n">
-        <v>-0.1492615920180186</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -526,9 +509,6 @@
       <c r="C6" t="n">
         <v>0.04048036993039651</v>
       </c>
-      <c r="D6" t="n">
-        <v>-0.01084470676710231</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -542,9 +522,6 @@
       <c r="C7" t="n">
         <v>0.6023352625551549</v>
       </c>
-      <c r="D7" t="n">
-        <v>-0.2890100199581167</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -558,9 +535,6 @@
       <c r="C8" t="n">
         <v>0.4635818182184269</v>
       </c>
-      <c r="D8" t="n">
-        <v>-0.1288068020067809</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -574,9 +548,6 @@
       <c r="C9" t="n">
         <v>0.04653574194719019</v>
       </c>
-      <c r="D9" t="n">
-        <v>-0.004967242491312236</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -590,9 +561,6 @@
       <c r="C10" t="n">
         <v>0.01329302213564387</v>
       </c>
-      <c r="D10" t="n">
-        <v>-0.007553950570012136</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -606,9 +574,6 @@
       <c r="C11" t="n">
         <v>0.01698016659525949</v>
       </c>
-      <c r="D11" t="n">
-        <v>0.005835982810582105</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -622,9 +587,6 @@
       <c r="C12" t="n">
         <v>-0.07078831792820627</v>
       </c>
-      <c r="D12" t="n">
-        <v>-0.1162453329140735</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -638,9 +600,6 @@
       <c r="C13" t="n">
         <v>0.2977445703353755</v>
       </c>
-      <c r="D13" t="n">
-        <v>0.5001672653568795</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
@@ -654,9 +613,6 @@
       <c r="C14" t="n">
         <v>-0.002773626894233351</v>
       </c>
-      <c r="D14" t="n">
-        <v>0.002185988857627289</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
@@ -670,9 +626,6 @@
       <c r="C15" t="n">
         <v>0.06867950143188847</v>
       </c>
-      <c r="D15" t="n">
-        <v>0.01265708164003366</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
@@ -686,9 +639,6 @@
       <c r="C16" t="n">
         <v>-0.1106956946134726</v>
       </c>
-      <c r="D16" t="n">
-        <v>-0.4541571688621455</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
@@ -702,9 +652,6 @@
       <c r="C17" t="n">
         <v>0.002172614347008018</v>
       </c>
-      <c r="D17" t="n">
-        <v>0.0007467146987063493</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
@@ -718,9 +665,6 @@
       <c r="C18" t="n">
         <v>0.1815311275614519</v>
       </c>
-      <c r="D18" t="n">
-        <v>-0.06476142820085663</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
@@ -734,9 +678,6 @@
       <c r="C19" t="n">
         <v>0.02929152104249704</v>
       </c>
-      <c r="D19" t="n">
-        <v>0.03618772585760481</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
@@ -750,9 +691,6 @@
       <c r="C20" t="n">
         <v>0.008555090637495428</v>
       </c>
-      <c r="D20" t="n">
-        <v>0.002940334043444173</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -765,9 +703,6 @@
       </c>
       <c r="C21" t="n">
         <v>0.1516615032275867</v>
-      </c>
-      <c r="D21" t="n">
-        <v>-0.0290212256805805</v>
       </c>
     </row>
   </sheetData>
@@ -781,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -795,11 +730,6 @@
           <t>PC2</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>PC3</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -813,9 +743,6 @@
       <c r="C2" t="n">
         <v>-0.1106956946134726</v>
       </c>
-      <c r="D2" t="n">
-        <v>-0.4541571688621455</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -829,9 +756,6 @@
       <c r="C3" t="n">
         <v>0.2977445703353755</v>
       </c>
-      <c r="D3" t="n">
-        <v>0.5001672653568795</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -845,56 +769,44 @@
       <c r="C4" t="n">
         <v>0.6023352625551549</v>
       </c>
-      <c r="D4" t="n">
-        <v>-0.2890100199581167</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Aluminium</t>
+          <t>Gold</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.113570768018911</v>
+        <v>-0.08346545507025413</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1743457149584367</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.633151850812806</v>
+        <v>0.4635818182184269</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Gold</t>
+          <t>Coal</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.08346545507025413</v>
+        <v>0.007881856112191934</v>
       </c>
       <c r="C6" t="n">
-        <v>0.4635818182184269</v>
-      </c>
-      <c r="D6" t="n">
-        <v>-0.1288068020067809</v>
+        <v>0.4642250012442724</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Coal</t>
+          <t>Aluminium</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.007881856112191934</v>
+        <v>0.113570768018911</v>
       </c>
       <c r="C7" t="n">
-        <v>0.4642250012442724</v>
-      </c>
-      <c r="D7" t="n">
-        <v>-0.1492615920180186</v>
+        <v>0.1743457149584367</v>
       </c>
     </row>
     <row r="8">
@@ -909,40 +821,31 @@
       <c r="C8" t="n">
         <v>0.1815311275614519</v>
       </c>
-      <c r="D8" t="n">
-        <v>-0.06476142820085663</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Manganese</t>
+          <t>Zinc</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.015640278992709</v>
+        <v>0.001041085819784322</v>
       </c>
       <c r="C9" t="n">
-        <v>-0.07078831792820627</v>
-      </c>
-      <c r="D9" t="n">
-        <v>-0.1162453329140735</v>
+        <v>0.1516615032275867</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Zinc</t>
+          <t>Manganese</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.001041085819784322</v>
+        <v>0.015640278992709</v>
       </c>
       <c r="C10" t="n">
-        <v>0.1516615032275867</v>
-      </c>
-      <c r="D10" t="n">
-        <v>-0.0290212256805805</v>
+        <v>-0.07078831792820627</v>
       </c>
     </row>
     <row r="11">
@@ -957,72 +860,57 @@
       <c r="C11" t="n">
         <v>0.06867950143188847</v>
       </c>
-      <c r="D11" t="n">
-        <v>0.01265708164003366</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>Tin</t>
+          <t>Bauxite</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.01397964134532832</v>
+        <v>-0.0008595630820294453</v>
       </c>
       <c r="C12" t="n">
-        <v>0.02929152104249704</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0.03618772585760481</v>
+        <v>0.06723050390707017</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Bauxite</t>
+          <t>Cobalt</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.0008595630820294453</v>
+        <v>-0.01658189283290847</v>
       </c>
       <c r="C13" t="n">
-        <v>0.06723050390707017</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0.002803927787755511</v>
+        <v>0.04048036993039651</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>Cobalt</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.01658189283290847</v>
+        <v>0.001985357329268395</v>
       </c>
       <c r="C14" t="n">
-        <v>0.04048036993039651</v>
-      </c>
-      <c r="D14" t="n">
-        <v>-0.01084470676710231</v>
+        <v>0.04653574194719019</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Tin</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.001985357329268395</v>
+        <v>-0.01397964134532832</v>
       </c>
       <c r="C15" t="n">
-        <v>0.04653574194719019</v>
-      </c>
-      <c r="D15" t="n">
-        <v>-0.004967242491312236</v>
+        <v>0.02929152104249704</v>
       </c>
     </row>
     <row r="16">
@@ -1037,9 +925,6 @@
       <c r="C16" t="n">
         <v>0.01698016659525949</v>
       </c>
-      <c r="D16" t="n">
-        <v>0.005835982810582105</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
@@ -1053,9 +938,6 @@
       <c r="C17" t="n">
         <v>0.01329302213564387</v>
       </c>
-      <c r="D17" t="n">
-        <v>-0.007553950570012136</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
@@ -1069,9 +951,6 @@
       <c r="C18" t="n">
         <v>0.008555090637495428</v>
       </c>
-      <c r="D18" t="n">
-        <v>0.002940334043444173</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
@@ -1085,9 +964,6 @@
       <c r="C19" t="n">
         <v>0.007877734388425772</v>
       </c>
-      <c r="D19" t="n">
-        <v>-0.004631330211285094</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
@@ -1101,9 +977,6 @@
       <c r="C20" t="n">
         <v>-0.002773626894233351</v>
       </c>
-      <c r="D20" t="n">
-        <v>0.002185988857627289</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -1116,9 +989,6 @@
       </c>
       <c r="C21" t="n">
         <v>0.002172614347008018</v>
-      </c>
-      <c r="D21" t="n">
-        <v>0.0007467146987063493</v>
       </c>
     </row>
   </sheetData>
@@ -1132,7 +1002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1151,11 +1021,6 @@
           <t>PC2</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>PC3</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -1164,13 +1029,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4.442677472228935</v>
+        <v>-2.921834852851945</v>
       </c>
       <c r="C2" t="n">
-        <v>0.6431398196761821</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.8059591884147032</v>
+        <v>3.749844358185245</v>
       </c>
     </row>
     <row r="3">
@@ -1180,13 +1042,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.149803002306768</v>
+        <v>1.624856762655432</v>
       </c>
       <c r="C3" t="n">
-        <v>-1.889900573076203</v>
-      </c>
-      <c r="D3" t="n">
-        <v>-1.79675837443147</v>
+        <v>-0.7730517261989613</v>
       </c>
     </row>
     <row r="4">
@@ -1196,13 +1055,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-3.371869522102026</v>
+        <v>5.482788157550414</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.9098187612605766</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.6534504270530082</v>
+        <v>0.4133279818826018</v>
       </c>
     </row>
     <row r="5">
@@ -1212,13 +1068,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-3.072725601102041</v>
+        <v>-3.323187591758097</v>
       </c>
       <c r="C5" t="n">
-        <v>4.04535057473371</v>
-      </c>
-      <c r="D5" t="n">
-        <v>-1.76658156237115</v>
+        <v>-1.057958692465072</v>
       </c>
     </row>
   </sheetData>
@@ -1232,7 +1085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1251,11 +1104,6 @@
           <t>PC2</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>PC3</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -1264,13 +1112,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.153271488754729</v>
+        <v>2.304406284324114</v>
       </c>
       <c r="C2" t="n">
-        <v>1.772734598624978</v>
-      </c>
-      <c r="D2" t="n">
-        <v>2.291882933890302</v>
+        <v>1.722384042962235</v>
       </c>
     </row>
     <row r="3">
@@ -1280,13 +1125,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.15760487097993</v>
+        <v>0.8506513211199691</v>
       </c>
       <c r="C3" t="n">
-        <v>0.6056891472229381</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.9271732698952012</v>
+        <v>2.02093751779211</v>
       </c>
     </row>
     <row r="4">
@@ -1296,13 +1138,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3677219092106317</v>
+        <v>1.58157230338235</v>
       </c>
       <c r="C4" t="n">
-        <v>0.8819579451065671</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.530681853314511</v>
+        <v>1.721311657971124</v>
       </c>
     </row>
     <row r="5">
@@ -1312,13 +1151,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.486180733063504</v>
+        <v>0.5670348141895912</v>
       </c>
       <c r="C5" t="n">
-        <v>1.681192192458464</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.7864740970669711</v>
+        <v>0.5625801186415249</v>
       </c>
     </row>
   </sheetData>
@@ -1354,7 +1190,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -1364,7 +1200,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -1374,7 +1210,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -1384,7 +1220,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1398,7 +1234,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1430,7 +1266,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4.442677472228935</v>
+        <v>-2.921834852851945</v>
       </c>
     </row>
     <row r="3">
@@ -1445,7 +1281,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.149803002306768</v>
+        <v>1.624856762655432</v>
       </c>
     </row>
     <row r="4">
@@ -1460,7 +1296,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>-3.371869522102026</v>
+        <v>5.482788157550414</v>
       </c>
     </row>
     <row r="5">
@@ -1475,7 +1311,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>-3.072725601102041</v>
+        <v>-3.323187591758097</v>
       </c>
     </row>
     <row r="6">
@@ -1490,7 +1326,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.6431398196761821</v>
+        <v>3.749844358185245</v>
       </c>
     </row>
     <row r="7">
@@ -1505,7 +1341,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>-1.889900573076203</v>
+        <v>-0.7730517261989613</v>
       </c>
     </row>
     <row r="8">
@@ -1520,7 +1356,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>-0.9098187612605766</v>
+        <v>0.4133279818826018</v>
       </c>
     </row>
     <row r="9">
@@ -1535,67 +1371,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>4.04535057473371</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>PC3</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>0.8059591884147032</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>PC3</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>-1.79675837443147</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>PC3</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>0.6534504270530082</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>PC3</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>-1.76658156237115</v>
+        <v>-1.057958692465072</v>
       </c>
     </row>
   </sheetData>

</xml_diff>